<commit_message>
enc: update code program dan test
</commit_message>
<xml_diff>
--- a/backend/public/excel/Product.xlsx
+++ b/backend/public/excel/Product.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>No</t>
   </si>
@@ -40,6 +40,9 @@
     <t>Es Campur</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
     <t>10.000</t>
   </si>
   <si>
@@ -55,13 +58,16 @@
     <t>Kentang Goreng</t>
   </si>
   <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>12.000</t>
   </si>
   <si>
     <t>Nasi Goreng</t>
   </si>
   <si>
-    <t>4</t>
+    <t>3</t>
   </si>
   <si>
     <t>20.000</t>
@@ -70,7 +76,7 @@
     <t>Sate Ayam</t>
   </si>
   <si>
-    <t>7</t>
+    <t>13</t>
   </si>
   <si>
     <t>30.000</t>
@@ -79,10 +85,16 @@
     <t>Sate Kambing Muda</t>
   </si>
   <si>
-    <t>5</t>
+    <t>18</t>
   </si>
   <si>
     <t>50.000</t>
+  </si>
+  <si>
+    <t>Sample Product</t>
+  </si>
+  <si>
+    <t>100</t>
   </si>
 </sst>
 </file>
@@ -471,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -530,10 +542,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -541,13 +553,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -555,13 +567,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -569,13 +581,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -583,13 +595,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -597,13 +609,27 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>